<commit_message>
Youth and graduate unemployment from MoSPI's published rates; quotations attributed (v2.49.0)
Neither series matched a published source. graduateUnemployment read 26.5
to 31.0 for recent years against MoSPI's 13.0 for graduates aged 15+ in
2023-24; youthUnemployment ran 2.5 to 3 points high and put its peak in
2020. Both are now MoSPI PLFS usual-status rates from api.mospi.gov.in,
retrieved 2026-10-10, with the years MoSPI does not publish left null.

The analyses become "four times the overall rate" (13.0 against 3.2 on
the same measure) and "fallen from 17.8% to 9.9% since 2017-18". The
homepage tile shows the latest published graduate year. The three worker
quotations in the data stories are attributed to primary research.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fDLqQaEK3pyPuRCQ1yqxy
</commit_message>
<xml_diff>
--- a/downloads/dataset.xlsx
+++ b/downloads/dataset.xlsx
@@ -260,44 +260,32 @@
           <t>youthUnemployment</t>
         </is>
       </c>
-      <c r="L4">
-        <v>13.5</v>
-      </c>
-      <c r="M4">
-        <v>13.8</v>
-      </c>
-      <c r="N4">
-        <v>14.2</v>
-      </c>
       <c r="O4">
-        <v>15.6</v>
+        <v>17.8</v>
       </c>
       <c r="P4">
-        <v>16.1</v>
+        <v>17.3</v>
       </c>
       <c r="Q4">
-        <v>14.8</v>
+        <v>15.0</v>
       </c>
       <c r="R4">
-        <v>17.8</v>
+        <v>12.9</v>
       </c>
       <c r="S4">
-        <v>13.2</v>
+        <v>12.4</v>
       </c>
       <c r="T4">
-        <v>12.9</v>
+        <v>10.0</v>
       </c>
       <c r="U4">
-        <v>12.9</v>
+        <v>10.2</v>
       </c>
       <c r="V4">
-        <v>12.8</v>
+        <v>10.3</v>
       </c>
       <c r="W4">
-        <v>12.5</v>
-      </c>
-      <c r="X4">
-        <v>12.3</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="5">
@@ -306,44 +294,26 @@
           <t>graduateUnemployment</t>
         </is>
       </c>
-      <c r="L5">
-        <v>18.5</v>
-      </c>
-      <c r="M5">
-        <v>19.2</v>
-      </c>
-      <c r="N5">
-        <v>21.0</v>
-      </c>
       <c r="O5">
-        <v>23.5</v>
+        <v>17.2</v>
       </c>
       <c r="P5">
-        <v>25.0</v>
+        <v>16.9</v>
       </c>
       <c r="Q5">
-        <v>23.0</v>
+        <v>17.2</v>
       </c>
       <c r="R5">
-        <v>31.0</v>
+        <v>15.5</v>
       </c>
       <c r="S5">
-        <v>25.0</v>
+        <v>14.9</v>
       </c>
       <c r="T5">
-        <v>22.0</v>
+        <v>13.4</v>
       </c>
       <c r="U5">
-        <v>29.1</v>
-      </c>
-      <c r="V5">
-        <v>28.5</v>
-      </c>
-      <c r="W5">
-        <v>27.0</v>
-      </c>
-      <c r="X5">
-        <v>26.5</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Formal employment and income shares corrected to the published figures (v2.50.0)
Inequality prose follows the World Inequality Lab table: top 1% 22.6% in
2022-23, bottom 50% 15.0%, no figure after 2022. 'Twelve straight years'
withdrawn. Primer 1951 and 1982 shares, the bottom 50% wealth share (6.4)
and the media-kit timeline corrected; an unsourced CMIE robustness row
removed. Release notes, version 2.50.0, rebuilt paper and site.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fDLqQaEK3pyPuRCQ1yqxy
</commit_message>
<xml_diff>
--- a/downloads/dataset.xlsx
+++ b/downloads/dataset.xlsx
@@ -323,34 +323,34 @@
         </is>
       </c>
       <c r="B6">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="C6">
-        <v>18.8</v>
+        <v>19.3</v>
       </c>
       <c r="D6">
-        <v>19.6</v>
+        <v>19.7</v>
       </c>
       <c r="E6">
         <v>20.1</v>
       </c>
       <c r="F6">
-        <v>20.5</v>
+        <v>20.4</v>
       </c>
       <c r="G6">
-        <v>20.6</v>
+        <v>20.8</v>
       </c>
       <c r="H6">
-        <v>21.0</v>
+        <v>21.2</v>
       </c>
       <c r="I6">
+        <v>21.1</v>
+      </c>
+      <c r="J6">
         <v>21.3</v>
       </c>
-      <c r="J6">
-        <v>21.0</v>
-      </c>
       <c r="K6">
-        <v>21.2</v>
+        <v>21.6</v>
       </c>
       <c r="L6">
         <v>21.3</v>
@@ -359,38 +359,26 @@
         <v>21.7</v>
       </c>
       <c r="N6">
+        <v>22.2</v>
+      </c>
+      <c r="O6">
+        <v>22.3</v>
+      </c>
+      <c r="P6">
+        <v>22.4</v>
+      </c>
+      <c r="Q6">
+        <v>21.6</v>
+      </c>
+      <c r="R6">
         <v>21.5</v>
       </c>
-      <c r="O6">
-        <v>21.5</v>
-      </c>
-      <c r="P6">
+      <c r="S6">
         <v>21.7</v>
-      </c>
-      <c r="Q6">
-        <v>22.1</v>
-      </c>
-      <c r="R6">
-        <v>22.3</v>
-      </c>
-      <c r="S6">
-        <v>22.5</v>
       </c>
       <c r="T6">
         <v>22.6</v>
       </c>
-      <c r="U6">
-        <v>22.6</v>
-      </c>
-      <c r="V6">
-        <v>22.6</v>
-      </c>
-      <c r="W6">
-        <v>22.8</v>
-      </c>
-      <c r="X6">
-        <v>23.0</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -399,73 +387,61 @@
         </is>
       </c>
       <c r="B7">
+        <v>18.8</v>
+      </c>
+      <c r="C7">
+        <v>18.4</v>
+      </c>
+      <c r="D7">
+        <v>17.9</v>
+      </c>
+      <c r="E7">
+        <v>17.5</v>
+      </c>
+      <c r="F7">
+        <v>17.0</v>
+      </c>
+      <c r="G7">
         <v>16.5</v>
       </c>
-      <c r="C7">
-        <v>16.3</v>
-      </c>
-      <c r="D7">
+      <c r="H7">
         <v>16.0</v>
-      </c>
-      <c r="E7">
-        <v>15.8</v>
-      </c>
-      <c r="F7">
-        <v>15.6</v>
-      </c>
-      <c r="G7">
-        <v>15.5</v>
-      </c>
-      <c r="H7">
-        <v>15.4</v>
       </c>
       <c r="I7">
         <v>15.3</v>
       </c>
       <c r="J7">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
       <c r="K7">
-        <v>15.1</v>
+        <v>15.0</v>
       </c>
       <c r="L7">
+        <v>14.7</v>
+      </c>
+      <c r="M7">
+        <v>14.5</v>
+      </c>
+      <c r="N7">
+        <v>14.1</v>
+      </c>
+      <c r="O7">
+        <v>13.9</v>
+      </c>
+      <c r="P7">
+        <v>14.4</v>
+      </c>
+      <c r="Q7">
+        <v>14.7</v>
+      </c>
+      <c r="R7">
+        <v>15.5</v>
+      </c>
+      <c r="S7">
+        <v>15.4</v>
+      </c>
+      <c r="T7">
         <v>15.0</v>
-      </c>
-      <c r="M7">
-        <v>14.7</v>
-      </c>
-      <c r="N7">
-        <v>14.9</v>
-      </c>
-      <c r="O7">
-        <v>14.9</v>
-      </c>
-      <c r="P7">
-        <v>14.7</v>
-      </c>
-      <c r="Q7">
-        <v>13.5</v>
-      </c>
-      <c r="R7">
-        <v>13.3</v>
-      </c>
-      <c r="S7">
-        <v>13.1</v>
-      </c>
-      <c r="T7">
-        <v>13.1</v>
-      </c>
-      <c r="U7">
-        <v>13.1</v>
-      </c>
-      <c r="V7">
-        <v>13.1</v>
-      </c>
-      <c r="W7">
-        <v>13.0</v>
-      </c>
-      <c r="X7">
-        <v>12.9</v>
       </c>
     </row>
     <row r="8">
@@ -474,44 +450,26 @@
           <t>formalEmployment</t>
         </is>
       </c>
-      <c r="L8">
-        <v>13.0</v>
-      </c>
-      <c r="M8">
-        <v>12.8</v>
-      </c>
-      <c r="N8">
-        <v>12.5</v>
-      </c>
       <c r="O8">
-        <v>12.2</v>
+        <v>11.5</v>
       </c>
       <c r="P8">
-        <v>11.9</v>
+        <v>11.4</v>
       </c>
       <c r="Q8">
-        <v>11.6</v>
+        <v>10.5</v>
       </c>
       <c r="R8">
-        <v>11.4</v>
+        <v>9.7</v>
       </c>
       <c r="S8">
-        <v>11.5</v>
+        <v>10.1</v>
       </c>
       <c r="T8">
-        <v>11.3</v>
+        <v>9.6</v>
       </c>
       <c r="U8">
-        <v>11.2</v>
-      </c>
-      <c r="V8">
-        <v>11.2</v>
-      </c>
-      <c r="W8">
-        <v>11.0</v>
-      </c>
-      <c r="X8">
-        <v>10.9</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="9">
@@ -520,44 +478,26 @@
           <t>informalEmployment</t>
         </is>
       </c>
-      <c r="L9">
-        <v>87.0</v>
-      </c>
-      <c r="M9">
-        <v>87.2</v>
-      </c>
-      <c r="N9">
-        <v>87.5</v>
-      </c>
       <c r="O9">
-        <v>87.8</v>
+        <v>88.5</v>
       </c>
       <c r="P9">
-        <v>88.1</v>
+        <v>88.6</v>
       </c>
       <c r="Q9">
-        <v>88.4</v>
+        <v>89.5</v>
       </c>
       <c r="R9">
-        <v>88.6</v>
+        <v>90.3</v>
       </c>
       <c r="S9">
-        <v>88.5</v>
+        <v>89.9</v>
       </c>
       <c r="T9">
-        <v>88.7</v>
+        <v>90.4</v>
       </c>
       <c r="U9">
-        <v>88.8</v>
-      </c>
-      <c r="V9">
-        <v>88.8</v>
-      </c>
-      <c r="W9">
-        <v>89.0</v>
-      </c>
-      <c r="X9">
-        <v>89.1</v>
+        <v>89.9</v>
       </c>
     </row>
     <row r="10">
@@ -709,7 +649,7 @@
         <v>4.4</v>
       </c>
       <c r="X11">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="12">
@@ -831,7 +771,7 @@
         <v>87</v>
       </c>
       <c r="X13">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Indices, fiscal and jobs claims checked against their publishers (v2.51.0)
Master dataset written from the sources of record and checked in CI;
replication scripts rewritten to run against it and reproduce the
eight-of-nine comparison. Methodology document rewritten to describe
what the project does. Citizen-guide tax example and the direct-tax
claim sourced. NDA DQI average corrected to 0.37. Release notes,
version 2.51.0, rebuilt paper, site and dataset.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fDLqQaEK3pyPuRCQ1yqxy
</commit_message>
<xml_diff>
--- a/downloads/dataset.xlsx
+++ b/downloads/dataset.xlsx
@@ -531,7 +531,7 @@
         <v>131</v>
       </c>
       <c r="J10">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="K10">
         <v>140</v>
@@ -762,7 +762,7 @@
         <v>79</v>
       </c>
       <c r="U13">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="V13">
         <v>84</v>
@@ -847,7 +847,7 @@
         <v>6.55</v>
       </c>
       <c r="X14">
-        <v>6.4</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="15">
@@ -857,73 +857,73 @@
         </is>
       </c>
       <c r="B15">
-        <v>0.0</v>
+        <v>0.28</v>
       </c>
       <c r="C15">
-        <v>0.03</v>
+        <v>0.29</v>
       </c>
       <c r="D15">
-        <v>0.05</v>
+        <v>0.32</v>
       </c>
       <c r="E15">
-        <v>0.07</v>
+        <v>0.35</v>
       </c>
       <c r="F15">
-        <v>0.09</v>
+        <v>0.39</v>
       </c>
       <c r="G15">
-        <v>0.11</v>
+        <v>0.43</v>
       </c>
       <c r="H15">
-        <v>0.12</v>
+        <v>0.34</v>
       </c>
       <c r="I15">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="J15">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="K15">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="L15">
+        <v>0.42</v>
+      </c>
+      <c r="M15">
         <v>0.19</v>
       </c>
-      <c r="M15">
-        <v>0.21</v>
-      </c>
       <c r="N15">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="O15">
+        <v>0.36</v>
+      </c>
+      <c r="P15">
+        <v>0.38</v>
+      </c>
+      <c r="Q15">
+        <v>0.48</v>
+      </c>
+      <c r="R15">
+        <v>0.87</v>
+      </c>
+      <c r="S15">
+        <v>0.58</v>
+      </c>
+      <c r="T15">
+        <v>0.51</v>
+      </c>
+      <c r="U15">
+        <v>0.45</v>
+      </c>
+      <c r="V15">
+        <v>0.44</v>
+      </c>
+      <c r="W15">
         <v>0.41</v>
       </c>
-      <c r="P15">
-        <v>0.53</v>
-      </c>
-      <c r="Q15">
-        <v>0.65</v>
-      </c>
-      <c r="R15">
-        <v>0.92</v>
-      </c>
-      <c r="S15">
-        <v>0.82</v>
-      </c>
-      <c r="T15">
-        <v>0.7</v>
-      </c>
-      <c r="U15">
-        <v>0.68</v>
-      </c>
-      <c r="V15">
-        <v>0.68</v>
-      </c>
-      <c r="W15">
-        <v>0.68</v>
-      </c>
       <c r="X15">
-        <v>0.68</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="16">
@@ -948,7 +948,7 @@
         <v>0.58</v>
       </c>
       <c r="G16">
-        <v>0.61</v>
+        <v>0.6</v>
       </c>
       <c r="H16">
         <v>0.56</v>
@@ -957,7 +957,7 @@
         <v>0.54</v>
       </c>
       <c r="J16">
-        <v>0.51</v>
+        <v>0.53</v>
       </c>
       <c r="K16">
         <v>0.51</v>
@@ -999,7 +999,7 @@
         <v>0.3</v>
       </c>
       <c r="X16">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
A full fact check of every page (v2.52.0)
Every factual claim on the site, the paper, the walkthrough, the
explainers and the downloads checked against its source; corrections
applied file by file. Charts for the two deleted series removed; the
communal and sanitation charts relabelled to what they hold. The CI date
check now rejects stale data-vintage labels and lets dated events pass.
Release notes, version 2.52.0, rebuilt paper, site and dataset.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fDLqQaEK3pyPuRCQ1yqxy
</commit_message>
<xml_diff>
--- a/downloads/dataset.xlsx
+++ b/downloads/dataset.xlsx
@@ -142,10 +142,10 @@
         <v>7.9</v>
       </c>
       <c r="C2">
-        <v>9.3</v>
+        <v>7.9</v>
       </c>
       <c r="D2">
-        <v>9.3</v>
+        <v>8.1</v>
       </c>
       <c r="E2">
         <v>7.7</v>
@@ -175,36 +175,33 @@
         <v>8.0</v>
       </c>
       <c r="N2">
-        <v>8.2</v>
+        <v>8.3</v>
       </c>
       <c r="O2">
+        <v>6.8</v>
+      </c>
+      <c r="P2">
+        <v>6.5</v>
+      </c>
+      <c r="Q2">
+        <v>3.9</v>
+      </c>
+      <c r="R2">
+        <v>-5.8</v>
+      </c>
+      <c r="S2">
+        <v>9.7</v>
+      </c>
+      <c r="T2">
+        <v>7.6</v>
+      </c>
+      <c r="U2">
+        <v>7.3</v>
+      </c>
+      <c r="V2">
         <v>7.2</v>
       </c>
-      <c r="P2">
-        <v>6.1</v>
-      </c>
-      <c r="Q2">
-        <v>4.2</v>
-      </c>
-      <c r="R2">
-        <v>-7.3</v>
-      </c>
-      <c r="S2">
-        <v>8.7</v>
-      </c>
-      <c r="T2">
-        <v>7.2</v>
-      </c>
-      <c r="U2">
-        <v>7.6</v>
-      </c>
-      <c r="V2">
-        <v>7.8</v>
-      </c>
       <c r="W2">
-        <v>6.5</v>
-      </c>
-      <c r="X2">
         <v>7.8</v>
       </c>
     </row>
@@ -214,15 +211,9 @@
           <t>unemployment</t>
         </is>
       </c>
-      <c r="L3">
-        <v>4.9</v>
-      </c>
       <c r="M3">
         <v>5.0</v>
       </c>
-      <c r="N3">
-        <v>5.0</v>
-      </c>
       <c r="O3">
         <v>6.0</v>
       </c>
@@ -683,10 +674,10 @@
         <v>8.9</v>
       </c>
       <c r="J12">
-        <v>9.3</v>
+        <v>9.5</v>
       </c>
       <c r="K12">
-        <v>10.9</v>
+        <v>10.0</v>
       </c>
       <c r="L12">
         <v>6.7</v>
@@ -695,34 +686,34 @@
         <v>4.9</v>
       </c>
       <c r="N12">
-        <v>4.5</v>
+        <v>5.0</v>
       </c>
       <c r="O12">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
       <c r="P12">
-        <v>3.4</v>
+        <v>3.9</v>
       </c>
       <c r="Q12">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
       <c r="R12">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
       <c r="S12">
-        <v>5.5</v>
+        <v>5.1</v>
       </c>
       <c r="T12">
         <v>6.7</v>
       </c>
       <c r="U12">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="V12">
-        <v>4.6</v>
+        <v>4.9</v>
       </c>
       <c r="W12">
-        <v>4.0</v>
+        <v>2.2</v>
       </c>
       <c r="X12">
         <v>3.8</v>
@@ -820,16 +811,16 @@
         <v>1.05</v>
       </c>
       <c r="O14">
-        <v>2.05</v>
+        <v>1.05</v>
       </c>
       <c r="P14">
-        <v>4.0</v>
+        <v>1.8</v>
       </c>
       <c r="Q14">
-        <v>4.8</v>
+        <v>5.5</v>
       </c>
       <c r="R14">
-        <v>7.0</v>
+        <v>7.3</v>
       </c>
       <c r="S14">
         <v>9.0</v>

</xml_diff>

<commit_message>
Fact-check corrections, generated data pages and published forecasts (work in progress)
GDP 2023-25 and CPI 2025 corrected to MoSPI's releases; estimates block for
Budget Estimates and projections; analysis pages rebuilt with charts and
redirects; forecasts page; downloads and paper corrections; CI and docs
prepared for retiring the old dashboard.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fDLqQaEK3pyPuRCQ1yqxy
</commit_message>
<xml_diff>
--- a/downloads/dataset.xlsx
+++ b/downloads/dataset.xlsx
@@ -196,13 +196,13 @@
         <v>7.6</v>
       </c>
       <c r="U2">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="V2">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="W2">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="3">
@@ -639,9 +639,6 @@
       <c r="W11">
         <v>4.4</v>
       </c>
-      <c r="X11">
-        <v>4.3</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -713,7 +710,7 @@
         <v>4.9</v>
       </c>
       <c r="W12">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="X12">
         <v>3.8</v>
@@ -1007,9 +1004,6 @@
       </c>
       <c r="Q17">
         <v>6.8</v>
-      </c>
-      <c r="R17">
-        <v>7.7</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
September data and the IMF's October outlook (2.57.0)
- CPI inflation and unemployment for 2026 now average January to
  September (4.0% and 5.1%, from 3.8% and 5.2%), from MoSPI's API via
  tools/refresh_monthly.py. Youth unemployment on the monthly measure
  averages 15.3%, checked against the eight-month 15.4% it replaces.
- The IMF row on the forecasts page carries the October 2026 WEO
  (Chapter 1, Table 1.1 and Annex Table 1.1.2): 7.0% for 2026-27 and
  2027-28, CPI 5.0%. The sentence calling the IMF the low outlier is now
  computed from the rows.
- The front page's CPI note takes its month range from the source note,
  so it no longer goes stale each month.
- Paper, primer, inflation explainer and technical appendix updated to
  the new figures; NDA CPI average 4.83%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014fDLqQaEK3pyPuRCQ1yqxy
</commit_message>
<xml_diff>
--- a/downloads/dataset.xlsx
+++ b/downloads/dataset.xlsx
@@ -242,7 +242,7 @@
         <v>3.1</v>
       </c>
       <c r="X3">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="4">
@@ -713,7 +713,7 @@
         <v>2.4</v>
       </c>
       <c r="X12">
-        <v>3.8</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="13">

</xml_diff>